<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-14 06:32
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92702C67-0FD4-4B7D-AF21-EF95385FEFD8}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4CE20EE7-E3DA-405C-8133-B8A51713B4EF}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F42E151D-750B-459C-96D6-41FCA0CFF83E}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-15 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C4DFC9E-8176-4CDF-A91E-D36E49066EE1}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76271C3B-6B9A-49C2-A08A-E77642183CB6}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98B79042-351A-452C-824E-FBDF010A0D0B}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-16 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28791961-BD52-4D6A-AF4C-2E59F69032A8}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{749F9DBE-E4D1-46EA-BE8E-176D775640B4}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4ED2200-AA92-43C6-BA0C-A03D2E4E84D8}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-17 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3302FE35-A9BD-4035-A1D5-6E5367E072A9}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2CE8377-8E11-461B-9547-CF094DA14367}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0136688B-4610-45AF-859A-5B802095DE51}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-18 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D26BF95A-43CA-4568-9DA7-5A6DF5446B79}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0021218C-751D-4994-9592-9E5B6BE2FE5B}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EA72EE7-E3C4-45CE-90A5-84E674A89DD2}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-21 06:32
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98134DFC-9C7F-4F91-8C9A-03146AE1A1B7}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D03BA1F6-C27A-46A3-B460-6DC7BFC36AB6}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2EF6E36F-DFA6-4C75-8C30-E4069DA2BD16}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-22 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7516,4 +7516,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{09C8D40A-3371-4AF7-83C0-C27A0FA79598}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E09A5321-6F7C-446B-ACD1-BB5AC82E8694}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4E6B1B0-FA67-4DEC-A663-5AB0C8F538BD}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-23 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A209656-EA46-4186-ABC5-2007DCFB0327}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84E41DD1-7DDB-4C71-BE49-7A9CA08B8733}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0EA3D649-75B9-4528-AB37-30AE75F2E46D}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-24 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D023554-40DF-4EA4-859C-B84CC3DFAD81}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08002B98-DB9F-4C83-AFEF-EC4EAA18A263}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AEDA619B-7ADA-405D-975C-DFAA2EE81B0D}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-25 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA71D68D-ADE0-40B7-9E76-C920E4478FDB}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C9543BD6-9640-4573-B3D2-51B4B063FD13}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AB248A9-D2E1-479D-A485-E992A1201700}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-28 06:42
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8002310C-09B6-4F3A-9A17-A3AC87D9AF34}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DA27D83-C0F5-409E-AC88-50C71A081BA0}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECA3CFED-5911-47DA-88D2-A850AFBD80E2}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-29 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB8D533A-51BD-4598-8842-D0D83401CA50}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{09C5D2B3-B790-4294-8B88-B787F78A9D55}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2BEB9C0-4F54-4DEF-9F0B-E4C57EE16291}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-30 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{027FB161-02E4-4FBE-87D9-CFB3A7516314}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12AA8DF3-FFD0-4F48-A89E-4AD1F5593344}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98CF0916-3CB9-4F51-AB28-263B9030B715}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-01 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2AD5CE5F-71BA-4478-ADAA-F87D4301E950}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C83A4DD0-7B5D-4B67-9709-F5F9AABFBA30}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E82DDFD1-ABBC-480C-BC52-94367E567981}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-02 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{109B9E8D-4463-47D1-BC84-BEA3EF15A585}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6C97AE3-DEF4-41DD-B181-A6B99CDC402F}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7AC3B1BC-4BBA-4373-8DF1-E16162F94B06}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-05 06:32
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D715450-096F-449D-A8CF-DCEDFC918F51}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3177F566-83A8-468D-812D-DB82BC66FF95}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E35D9C60-687F-4D8C-939D-BD073BE5E2EF}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-06 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9827567-C26E-4A36-9154-9F27335FED30}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0945AFF9-235A-457F-8FC1-D1ABD9041370}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B871549-7044-4B71-96A2-46FE1E5715E7}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-07 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2A54AEB-19BD-4B44-A6FE-7B73E6FBE3BB}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{759232D3-F22F-45C2-940B-38FB4961B50C}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76B3E91E-5A3E-45E3-BAD6-E2FD087000D7}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-08 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D56D2048-6B8B-40CF-BC07-50F20B138AFE}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7193B7BA-5742-4517-A4F9-FF053E8F2B56}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6DAF5EA-467B-43B8-829D-B42A6F74861F}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-09 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E250DA5B-6E99-449F-A5B1-C8D5BB273AFA}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2CA2B38-E7CA-41E1-9971-1E8BB33417BF}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{59DC2CD5-DEA2-4309-902F-8DD37FBDBBDA}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-12 06:42
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFCF1F92-B84A-4C8B-98F8-F46827F507BA}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C6174CD-D900-4B36-9B9E-333C51E8336D}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C86FD817-328D-4326-AA2F-16920F83C2CC}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-13 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{915ECBDB-C090-4A99-BD13-D8D36E8E5257}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FE223A9-D639-4364-A9CD-834A490261F6}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D6CDD5F-5CD1-46C5-B464-EFAF84597927}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-15 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23A1109E-8D5D-4519-8D13-E1604309FADE}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{572982BE-3A07-4C5A-AFD4-CC4785554CE2}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9CAD105E-2350-4B49-AA93-B72B00EC564B}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-16 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7446,4 +7446,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E124FC9-B218-4010-B9F8-C5A5D490B91E}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02E523A9-26B1-42A6-9F5D-77525BAF7B56}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D128208A-FAD0-40DC-A2EB-6C17AFE4D008}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-19 06:33
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7446,4 +7446,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{581FB2AA-AC21-4530-A5B0-CCAE80CE4B6B}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEA6E291-7F36-417C-8D8F-3FE58641E332}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E38C25DB-0CB6-434E-9AAD-39FA25B7E35F}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-20 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7446,4 +7446,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CACD5E07-2765-4EFC-8CC8-DC708707C2DB}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F9D9743-CCB4-4A0B-9310-C1BD30DA0293}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26F3B022-3478-4F94-AF92-147932E948F1}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-21 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7446,4 +7446,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D17C597D-B430-4554-B504-FC504B2E2BC6}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F97FAA65-3AEA-4CFA-984A-60AAC4F4E0E8}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D9E6FFE-89FB-44E6-9B47-CA575DA6C79A}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-22 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7446,4 +7446,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0CC721C-993C-4524-8C66-ED7D5631C14E}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{365D7988-5104-43AA-9031-014FA6254467}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CD7572-2930-4C57-8562-5F27F51282F6}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-23 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7446,4 +7446,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{915419CB-F7DE-4AD1-AA49-99ACFC1BF1BD}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD6E5E55-3CB5-42CC-A83F-78339D6D5673}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E38ED409-F538-4684-BD07-D45124D27C85}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-26 06:37
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7446,4 +7446,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C3DB18F-B8A8-466C-982C-089A5CF9D822}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BADB5AF-A244-4AA8-9376-BC12DDA771B1}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD1DD7D7-F75C-42E0-9D34-24D5814C37D5}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-27 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7446,4 +7446,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{691C8E76-47EB-43A9-9F88-8353FCFDEDBF}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D577787-7CE8-45AB-95B5-AA5A213DCDD5}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EAA47D3-7072-4968-BAAD-4C8791D6F531}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-28 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7446,4 +7446,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{410EE7DD-2C5D-409E-A524-9E70C1C8B113}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39BC00C7-AC74-43A1-8A49-A3863F111C0B}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3590DF47-D510-4B65-885A-ECCBA3F6BAFE}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-29 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7446,4 +7446,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4513CB4-D2A4-4592-BE25-D34DC5E5A337}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F0531B1-0525-4D95-8090-88508BD8B6D6}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48B19D35-0B13-4E6D-BD5A-92D601EE22FD}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-10-30 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7446,4 +7446,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D96A8388-C158-40AE-8CB4-43679ABB2304}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0CA3938-0E78-4484-9406-AC3E722643D9}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{649BB22B-9A0D-403F-9C77-BB9142D23C2A}"/>
 </file>
</xml_diff>